<commit_message>
Add word "beskytte" to Repeats.xlsx
</commit_message>
<xml_diff>
--- a/sets/Repeats.xlsx
+++ b/sets/Repeats.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -517,9 +517,95 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>49a9c655-f892-440d-b53e-3bf3b6965ce6</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>beskytte</v>
+      </c>
+      <c r="D2" t="str">
+        <v>beskytte</v>
+      </c>
+      <c r="E2" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[beˈsgødə]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004239_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>forhindre at nogen eller noget lider skade eller overlast; sikre mod at nogen kommer i fare, i nød eller i en anden uønsket situation</v>
+      </c>
+      <c r="K2" t="str">
+        <v>protect</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -528,28 +614,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -631,8 +717,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Phone: progress 1, log 2 in Repeats.xlsx
</commit_message>
<xml_diff>
--- a/sets/Repeats.xlsx
+++ b/sets/Repeats.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Words" sheetId="1" r:id="rId1"/>
     <sheet name="Phrases" sheetId="2" r:id="rId2"/>
     <sheet name="Meta" sheetId="3" r:id="rId3"/>
+    <sheet name="ReviewLog" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -123,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,36 +400,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AH2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +523,24 @@
       <c r="AB1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="AC1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -573,19 +598,19 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>2026-07-21</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X2" t="str">
         <v/>
@@ -601,18 +626,27 @@
       </c>
       <c r="AB2" t="str">
         <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v>0.34</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>7.63</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:AB1"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="10.83203125"/>
     <col min="2" max="2" customWidth="1" width="11.83203125"/>
@@ -636,6 +670,12 @@
     <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
     <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
     <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,10 +745,28 @@
       <c r="V1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="W1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -758,4 +816,103 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Dir</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Grade</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Elapsed</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Interval</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>49a9c655-f892-440d-b53e-3bf3b6965ce6</v>
+      </c>
+      <c r="B2" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-07-20T10:30:02.126Z</v>
+      </c>
+      <c r="D2" t="str">
+        <v>again</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G2" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H2" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>49a9c655-f892-440d-b53e-3bf3b6965ce6</v>
+      </c>
+      <c r="B3" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-07-20T10:30:06.692Z</v>
+      </c>
+      <c r="D3" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E3" t="str">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>0.34</v>
+      </c>
+      <c r="G3" t="str">
+        <v>7.63</v>
+      </c>
+      <c r="H3" t="str">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 1, log 1 in Repeats.xlsx
</commit_message>
<xml_diff>
--- a/sets/Repeats.xlsx
+++ b/sets/Repeats.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -598,7 +598,7 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T2" t="str">
         <v>1</v>
@@ -607,7 +607,7 @@
         <v>2.5</v>
       </c>
       <c r="V2" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W2" t="str">
         <v>1</v>
@@ -628,13 +628,13 @@
         <v/>
       </c>
       <c r="AC2" t="str">
-        <v>0.48</v>
+        <v>0.76</v>
       </c>
       <c r="AD2" t="str">
-        <v>8.36</v>
+        <v>8.6</v>
       </c>
       <c r="AE2" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-25</v>
       </c>
     </row>
   </sheetData>
@@ -820,7 +820,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -962,9 +962,35 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>49a9c655-f892-440d-b53e-3bf3b6965ce6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-07-25T06:20:39.407Z</v>
+      </c>
+      <c r="D6" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E6" t="str">
+        <v>1</v>
+      </c>
+      <c r="F6" t="str">
+        <v>0.76</v>
+      </c>
+      <c r="G6" t="str">
+        <v>8.6</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>